<commit_message>
style(sheets): 민요 검수 xlsx 가사 열 글꼴 18pt (xlsx_font.py LYRIC_SIZE 12 → 18)
</commit_message>
<xml_diff>
--- a/sheets/민요/검수/각설이 타령.xlsx
+++ b/sheets/민요/검수/각설이 타령.xlsx
@@ -652,7 +652,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <name val="궁서체"/>
@@ -709,6 +709,12 @@
     <font>
       <b val="true"/>
       <sz val="24"/>
+      <name val="궁서체"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="18"/>
       <name val="궁서체"/>
       <family val="2"/>
       <charset val="1"/>
@@ -804,7 +810,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -906,6 +912,34 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5325,21 +5359,21 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="15" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="16" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="26" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="15" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="16" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="26" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="15" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="16" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="26" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="15" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="16" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="26" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="15" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="16" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="26" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="15" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="16" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="26" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="15" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="16" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="26" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="15" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="16" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="26" width="6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -5367,49 +5401,49 @@
       <c r="B3" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="27" t="s">
         <v>155</v>
       </c>
       <c r="D3" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="27" t="s">
         <v>138</v>
       </c>
       <c r="F3" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="27" t="s">
         <v>133</v>
       </c>
       <c r="H3" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="28" t="s">
         <v>125</v>
       </c>
       <c r="J3" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="K3" s="19" t="s">
+      <c r="K3" s="27" t="s">
         <v>115</v>
       </c>
       <c r="L3" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="M3" s="19" t="s">
+      <c r="M3" s="27" t="s">
         <v>98</v>
       </c>
       <c r="N3" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="O3" s="19" t="s">
+      <c r="O3" s="27" t="s">
         <v>81</v>
       </c>
       <c r="P3" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="Q3" s="19" t="s">
+      <c r="Q3" s="27" t="s">
         <v>46</v>
       </c>
     </row>
@@ -5417,49 +5451,49 @@
       <c r="B4" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="29" t="s">
         <v>156</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="29" t="s">
         <v>143</v>
       </c>
       <c r="F4" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="G4" s="29" t="s">
         <v>166</v>
       </c>
       <c r="H4" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="I4" s="22" t="s">
+      <c r="I4" s="29" t="s">
         <v>99</v>
       </c>
       <c r="J4" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="K4" s="22" t="s">
+      <c r="K4" s="29" t="s">
         <v>116</v>
       </c>
       <c r="L4" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="M4" s="22" t="s">
+      <c r="M4" s="29" t="s">
         <v>99</v>
       </c>
       <c r="N4" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="O4" s="22" t="s">
+      <c r="O4" s="29" t="s">
         <v>167</v>
       </c>
       <c r="P4" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="Q4" s="22" t="s">
+      <c r="Q4" s="29" t="s">
         <v>168</v>
       </c>
     </row>
@@ -5467,49 +5501,49 @@
       <c r="B5" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="29" t="s">
         <v>157</v>
       </c>
       <c r="D5" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="30" t="s">
         <v>144</v>
       </c>
       <c r="F5" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="G5" s="22" t="s">
+      <c r="G5" s="29" t="s">
         <v>133</v>
       </c>
       <c r="H5" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="I5" s="22" t="s">
+      <c r="I5" s="29" t="s">
         <v>100</v>
       </c>
       <c r="J5" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="K5" s="22" t="s">
+      <c r="K5" s="29" t="s">
         <v>117</v>
       </c>
       <c r="L5" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="M5" s="22" t="s">
+      <c r="M5" s="29" t="s">
         <v>100</v>
       </c>
       <c r="N5" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="O5" s="22" t="s">
+      <c r="O5" s="29" t="s">
         <v>81</v>
       </c>
       <c r="P5" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="Q5" s="22" t="s">
+      <c r="Q5" s="29" t="s">
         <v>51</v>
       </c>
     </row>
@@ -5517,49 +5551,49 @@
       <c r="B6" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="31" t="s">
         <v>169</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="31" t="s">
         <v>143</v>
       </c>
       <c r="F6" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="24" t="s">
+      <c r="G6" s="31" t="s">
         <v>166</v>
       </c>
       <c r="H6" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="I6" s="24" t="s">
+      <c r="I6" s="31" t="s">
         <v>101</v>
       </c>
       <c r="J6" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="K6" s="24" t="s">
+      <c r="K6" s="31" t="s">
         <v>170</v>
       </c>
       <c r="L6" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="M6" s="24" t="s">
+      <c r="M6" s="31" t="s">
         <v>101</v>
       </c>
       <c r="N6" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="O6" s="24" t="s">
+      <c r="O6" s="31" t="s">
         <v>171</v>
       </c>
       <c r="P6" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="Q6" s="24" t="s">
+      <c r="Q6" s="31" t="s">
         <v>172</v>
       </c>
     </row>
@@ -5567,49 +5601,49 @@
       <c r="B7" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="27" t="s">
         <v>173</v>
       </c>
       <c r="D7" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="27" t="s">
         <v>174</v>
       </c>
       <c r="F7" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="27" t="s">
         <v>133</v>
       </c>
       <c r="H7" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="I7" s="19" t="s">
+      <c r="I7" s="27" t="s">
         <v>125</v>
       </c>
       <c r="J7" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="K7" s="19" t="s">
+      <c r="K7" s="27" t="s">
         <v>175</v>
       </c>
       <c r="L7" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="M7" s="19" t="s">
+      <c r="M7" s="27" t="s">
         <v>67</v>
       </c>
       <c r="N7" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="O7" s="19" t="s">
+      <c r="O7" s="27" t="s">
         <v>176</v>
       </c>
       <c r="P7" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="Q7" s="19" t="s">
+      <c r="Q7" s="27" t="s">
         <v>53</v>
       </c>
     </row>
@@ -5617,49 +5651,49 @@
       <c r="B8" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="29" t="s">
         <v>177</v>
       </c>
       <c r="D8" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="29" t="s">
         <v>178</v>
       </c>
       <c r="F8" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="G8" s="22" t="s">
+      <c r="G8" s="29" t="s">
         <v>135</v>
       </c>
       <c r="H8" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="I8" s="22" t="s">
+      <c r="I8" s="29" t="s">
         <v>127</v>
       </c>
       <c r="J8" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="K8" s="22" t="s">
+      <c r="K8" s="29" t="s">
         <v>179</v>
       </c>
       <c r="L8" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="M8" s="22" t="s">
+      <c r="M8" s="29" t="s">
         <v>98</v>
       </c>
       <c r="N8" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="O8" s="22" t="s">
+      <c r="O8" s="29" t="s">
         <v>180</v>
       </c>
       <c r="P8" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="Q8" s="22" t="s">
+      <c r="Q8" s="29" t="s">
         <v>181</v>
       </c>
     </row>
@@ -5667,41 +5701,41 @@
       <c r="B9" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="C9" s="22"/>
+      <c r="C9" s="29"/>
       <c r="D9" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="E9" s="22"/>
+      <c r="E9" s="29"/>
       <c r="F9" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="22" t="s">
+      <c r="G9" s="29" t="s">
         <v>182</v>
       </c>
       <c r="H9" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="I9" s="22" t="s">
+      <c r="I9" s="29" t="s">
         <v>102</v>
       </c>
       <c r="J9" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="K9" s="22"/>
+      <c r="K9" s="29"/>
       <c r="L9" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="M9" s="22" t="s">
+      <c r="M9" s="29" t="s">
         <v>102</v>
       </c>
       <c r="N9" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="O9" s="22"/>
+      <c r="O9" s="29"/>
       <c r="P9" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="Q9" s="22" t="s">
+      <c r="Q9" s="29" t="s">
         <v>59</v>
       </c>
     </row>
@@ -5709,41 +5743,41 @@
       <c r="B10" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="C10" s="24"/>
+      <c r="C10" s="31"/>
       <c r="D10" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="E10" s="24"/>
+      <c r="E10" s="31"/>
       <c r="F10" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="G10" s="24" t="s">
+      <c r="G10" s="31" t="s">
         <v>183</v>
       </c>
       <c r="H10" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="I10" s="24" t="s">
+      <c r="I10" s="31" t="s">
         <v>103</v>
       </c>
       <c r="J10" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="K10" s="25"/>
+      <c r="K10" s="32"/>
       <c r="L10" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="M10" s="24" t="s">
+      <c r="M10" s="31" t="s">
         <v>103</v>
       </c>
       <c r="N10" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="O10" s="25"/>
+      <c r="O10" s="32"/>
       <c r="P10" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="Q10" s="24" t="s">
+      <c r="Q10" s="31" t="s">
         <v>60</v>
       </c>
     </row>
@@ -5751,49 +5785,49 @@
       <c r="B11" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="27" t="s">
         <v>184</v>
       </c>
       <c r="D11" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="27" t="s">
         <v>148</v>
       </c>
       <c r="F11" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="27" t="s">
         <v>138</v>
       </c>
       <c r="H11" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="I11" s="21" t="s">
+      <c r="I11" s="28" t="s">
         <v>128</v>
       </c>
       <c r="J11" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="K11" s="19" t="s">
+      <c r="K11" s="27" t="s">
         <v>123</v>
       </c>
       <c r="L11" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="M11" s="19" t="s">
+      <c r="M11" s="27" t="s">
         <v>104</v>
       </c>
       <c r="N11" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="O11" s="19" t="s">
+      <c r="O11" s="27" t="s">
         <v>96</v>
       </c>
       <c r="P11" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="Q11" s="19" t="s">
+      <c r="Q11" s="27" t="s">
         <v>46</v>
       </c>
     </row>
@@ -5801,47 +5835,47 @@
       <c r="B12" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="C12" s="22"/>
+      <c r="C12" s="29"/>
       <c r="D12" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="30" t="s">
         <v>149</v>
       </c>
       <c r="F12" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="G12" s="22" t="s">
+      <c r="G12" s="29" t="s">
         <v>139</v>
       </c>
       <c r="H12" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="I12" s="22" t="s">
+      <c r="I12" s="29" t="s">
         <v>130</v>
       </c>
       <c r="J12" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="K12" s="22" t="s">
+      <c r="K12" s="29" t="s">
         <v>185</v>
       </c>
       <c r="L12" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M12" s="22" t="s">
+      <c r="M12" s="29" t="s">
         <v>105</v>
       </c>
       <c r="N12" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="O12" s="22" t="s">
+      <c r="O12" s="29" t="s">
         <v>185</v>
       </c>
       <c r="P12" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="Q12" s="22" t="s">
+      <c r="Q12" s="29" t="s">
         <v>65</v>
       </c>
     </row>
@@ -5849,49 +5883,49 @@
       <c r="B13" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="29" t="s">
         <v>157</v>
       </c>
       <c r="D13" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="22" t="s">
+      <c r="E13" s="29" t="s">
         <v>151</v>
       </c>
       <c r="F13" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="29" t="s">
         <v>51</v>
       </c>
       <c r="H13" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="I13" s="22" t="s">
+      <c r="I13" s="29" t="s">
         <v>117</v>
       </c>
       <c r="J13" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="K13" s="22" t="s">
+      <c r="K13" s="29" t="s">
         <v>124</v>
       </c>
       <c r="L13" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="M13" s="22" t="s">
+      <c r="M13" s="29" t="s">
         <v>106</v>
       </c>
       <c r="N13" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="O13" s="22" t="s">
+      <c r="O13" s="29" t="s">
         <v>98</v>
       </c>
       <c r="P13" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="Q13" s="22" t="s">
+      <c r="Q13" s="29" t="s">
         <v>67</v>
       </c>
     </row>
@@ -5899,49 +5933,49 @@
       <c r="B14" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="31" t="s">
         <v>169</v>
       </c>
       <c r="D14" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="E14" s="24" t="s">
+      <c r="E14" s="31" t="s">
         <v>152</v>
       </c>
       <c r="F14" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G14" s="24" t="s">
+      <c r="G14" s="31" t="s">
         <v>186</v>
       </c>
       <c r="H14" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="I14" s="24" t="s">
+      <c r="I14" s="31" t="s">
         <v>170</v>
       </c>
       <c r="J14" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="K14" s="24" t="s">
+      <c r="K14" s="31" t="s">
         <v>168</v>
       </c>
       <c r="L14" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="M14" s="24" t="s">
+      <c r="M14" s="31" t="s">
         <v>107</v>
       </c>
       <c r="N14" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="O14" s="24" t="s">
+      <c r="O14" s="31" t="s">
         <v>168</v>
       </c>
       <c r="P14" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="Q14" s="24" t="s">
+      <c r="Q14" s="31" t="s">
         <v>70</v>
       </c>
     </row>
@@ -5949,49 +5983,49 @@
       <c r="B15" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="27" t="s">
         <v>173</v>
       </c>
       <c r="D15" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="27" t="s">
         <v>187</v>
       </c>
       <c r="F15" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="27" t="s">
         <v>133</v>
       </c>
       <c r="H15" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="I15" s="19" t="s">
+      <c r="I15" s="27" t="s">
         <v>175</v>
       </c>
       <c r="J15" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="K15" s="19" t="s">
+      <c r="K15" s="27" t="s">
         <v>53</v>
       </c>
       <c r="L15" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="M15" s="19" t="s">
+      <c r="M15" s="27" t="s">
         <v>188</v>
       </c>
       <c r="N15" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="O15" s="19" t="s">
+      <c r="O15" s="27" t="s">
         <v>53</v>
       </c>
       <c r="P15" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="Q15" s="19" t="s">
+      <c r="Q15" s="27" t="s">
         <v>72</v>
       </c>
     </row>
@@ -5999,49 +6033,49 @@
       <c r="B16" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="30" t="s">
         <v>189</v>
       </c>
       <c r="D16" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="E16" s="22" t="s">
+      <c r="E16" s="29" t="s">
         <v>190</v>
       </c>
       <c r="F16" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="G16" s="22" t="s">
+      <c r="G16" s="29" t="s">
         <v>135</v>
       </c>
       <c r="H16" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="I16" s="22" t="s">
+      <c r="I16" s="29" t="s">
         <v>179</v>
       </c>
       <c r="J16" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="K16" s="22" t="s">
+      <c r="K16" s="29" t="s">
         <v>181</v>
       </c>
       <c r="L16" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="M16" s="22" t="s">
+      <c r="M16" s="29" t="s">
         <v>191</v>
       </c>
       <c r="N16" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="O16" s="22" t="s">
+      <c r="O16" s="29" t="s">
         <v>181</v>
       </c>
       <c r="P16" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="Q16" s="22" t="s">
+      <c r="Q16" s="29" t="s">
         <v>75</v>
       </c>
     </row>
@@ -6049,41 +6083,41 @@
       <c r="B17" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="22"/>
+      <c r="C17" s="29"/>
       <c r="D17" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="E17" s="22"/>
+      <c r="E17" s="29"/>
       <c r="F17" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="G17" s="22" t="s">
+      <c r="G17" s="29" t="s">
         <v>141</v>
       </c>
       <c r="H17" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="I17" s="22"/>
+      <c r="I17" s="29"/>
       <c r="J17" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K17" s="22" t="s">
+      <c r="K17" s="29" t="s">
         <v>59</v>
       </c>
       <c r="L17" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="M17" s="23"/>
+      <c r="M17" s="30"/>
       <c r="N17" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="O17" s="22" t="s">
+      <c r="O17" s="29" t="s">
         <v>59</v>
       </c>
       <c r="P17" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="Q17" s="22" t="s">
+      <c r="Q17" s="29" t="s">
         <v>77</v>
       </c>
     </row>
@@ -6091,41 +6125,41 @@
       <c r="B18" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="C18" s="24"/>
+      <c r="C18" s="31"/>
       <c r="D18" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="E18" s="24"/>
+      <c r="E18" s="31"/>
       <c r="F18" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="G18" s="24" t="s">
+      <c r="G18" s="31" t="s">
         <v>142</v>
       </c>
       <c r="H18" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="I18" s="24"/>
+      <c r="I18" s="31"/>
       <c r="J18" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="K18" s="24" t="s">
+      <c r="K18" s="31" t="s">
         <v>60</v>
       </c>
       <c r="L18" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="M18" s="25"/>
+      <c r="M18" s="32"/>
       <c r="N18" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="O18" s="24" t="s">
+      <c r="O18" s="31" t="s">
         <v>60</v>
       </c>
       <c r="P18" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="Q18" s="24" t="s">
+      <c r="Q18" s="31" t="s">
         <v>80</v>
       </c>
     </row>

</xml_diff>

<commit_message>
style(sheets): 민요 검수 xlsx 아이보리(FFF2CC) 배경 제거 (94곡)
</commit_message>
<xml_diff>
--- a/sheets/민요/검수/각설이 타령.xlsx
+++ b/sheets/민요/검수/각설이 타령.xlsx
@@ -734,10 +734,7 @@
       </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
+      <patternFill patternType="none"/>
     </fill>
   </fills>
   <borders count="5">

</xml_diff>